<commit_message>
Pilot B: fix TEXTSPLIT #NAME? in fixture (missing _xlfn. prefix)
openpyxl writes newer dynamic-array functions (TEXTSPLIT, XLOOKUP, etc.)
without the internal _xlfn. prefix Excel needs to resolve the function
name. Without it, Excel shows #NAME? on every TEXTSPLIT formula and
displays it with a spurious leading @ (implicit intersection), even
though the formula text looks correct in the formula bar. Fixed by
writing the 4 TEXTSPLIT formulas as =_xlfn.TEXTSPLIT(...); confirmed
via Excel Online that this resolves and spills correctly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UjdUwHhnA5G4VgoVNxTMeX
</commit_message>
<xml_diff>
--- a/fixtures/excel-split-comma-values-into-rows_fixture.xlsx
+++ b/fixtures/excel-split-comma-values-into-rows_fixture.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="C2">
-        <f>TEXTSPLIT(B2,",")</f>
+        <f>_xlfn.TEXTSPLIT(B2,",")</f>
         <v/>
       </c>
     </row>
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="C5">
-        <f>TEXTSPLIT(B5,",",,FALSE)</f>
+        <f>_xlfn.TEXTSPLIT(B5,",",,FALSE)</f>
         <v/>
       </c>
     </row>
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="F6">
-        <f>TEXTSPLIT(B6,",",,TRUE)</f>
+        <f>_xlfn.TEXTSPLIT(B6,",",,TRUE)</f>
         <v/>
       </c>
     </row>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="C9">
-        <f>TEXTSPLIT(B9,{",",";"})</f>
+        <f>_xlfn.TEXTSPLIT(B9,{",",";"})</f>
         <v/>
       </c>
     </row>

</xml_diff>